<commit_message>
Write one workbook per pathway step and figures as S1-S19 pages
</commit_message>
<xml_diff>
--- a/03_Pathway_Enrichment/03_enrich_scatter_fgsea/c_data/03_enrich_scatter_fgsea.xlsx
+++ b/03_Pathway_Enrichment/03_enrich_scatter_fgsea/c_data/03_enrich_scatter_fgsea.xlsx
@@ -7,11 +7,10 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="concordance" sheetId="1" r:id="rId1"/>
-    <sheet name="discordant" sheetId="2" r:id="rId2"/>
-    <sheet name="nes_scatter" sheetId="3" r:id="rId3"/>
-    <sheet name="input_manifest" sheetId="4" r:id="rId4"/>
-    <sheet name="package_versions" sheetId="5" r:id="rId5"/>
+    <sheet name="overview" sheetId="1" r:id="rId1"/>
+    <sheet name="concordance" sheetId="2" r:id="rId2"/>
+    <sheet name="discordant" sheetId="3" r:id="rId3"/>
+    <sheet name="nes_scatter" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -355,119 +354,83 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>population</t>
+          <t>sheet</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>sets</t>
+          <t>rows</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>significant</t>
+          <t>columns</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>discordant</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>rho</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>p</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>same_sign</t>
+          <t>description</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>all collections</t>
+          <t>concordance</t>
         </is>
       </c>
       <c r="B2">
-        <v>1990</v>
+        <v>3</v>
       </c>
       <c r="C2">
-        <v>418</v>
-      </c>
-      <c r="D2">
-        <v>8</v>
-      </c>
-      <c r="E2">
-        <v>0.827</v>
-      </c>
-      <c r="F2">
-        <v>0</v>
-      </c>
-      <c r="G2">
-        <v>0.981</v>
+        <v>7</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Spearman rho and sign agreement of NES between the two training contrasts, per population</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>collapse survivors</t>
+          <t>discordant</t>
         </is>
       </c>
       <c r="B3">
-        <v>126</v>
+        <v>8</v>
       </c>
       <c r="C3">
-        <v>126</v>
-      </c>
-      <c r="D3">
-        <v>3</v>
-      </c>
-      <c r="E3">
-        <v>0.861</v>
-      </c>
-      <c r="F3">
-        <v>0</v>
-      </c>
-      <c r="G3">
-        <v>0.976</v>
+        <v>12</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Sets significant in one arm with NES of opposite sign in the other</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Hallmark and GO Slim</t>
+          <t>nes_scatter</t>
         </is>
       </c>
       <c r="B4">
-        <v>100</v>
+        <v>1990</v>
       </c>
       <c r="C4">
-        <v>25</v>
-      </c>
-      <c r="D4">
-        <v>0</v>
-      </c>
-      <c r="E4">
-        <v>0.8149999999999999</v>
-      </c>
-      <c r="F4">
-        <v>0</v>
-      </c>
-      <c r="G4">
-        <v>1</v>
+        <v>12</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Every set with its NES and adjusted p in both training contrasts</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -477,464 +440,118 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>set_id</t>
+          <t>population</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>database</t>
+          <t>sets</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>pathway</t>
+          <t>significant</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>label</t>
+          <t>discordant</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>genes</t>
+          <t>rho</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>nes_x</t>
+          <t>p</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>nes_y</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>padj_x</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>padj_y</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>significance</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>discordant</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>survivor</t>
+          <t>same_sign</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>GOBP|GOBP_SMALL_MOLECULE_CATABOLIC_PROCESS</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>GOBP</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>GOBP_SMALL_MOLECULE_CATABOLIC_PROCESS</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Small Molecule
-Catabolism</t>
-        </is>
+          <t>all collections</t>
+        </is>
+      </c>
+      <c r="B2">
+        <v>1990</v>
+      </c>
+      <c r="C2">
+        <v>418</v>
+      </c>
+      <c r="D2">
+        <v>8</v>
       </c>
       <c r="E2">
-        <v>157</v>
+        <v>0.827</v>
       </c>
       <c r="F2">
-        <v>1.725</v>
+        <v>0</v>
       </c>
       <c r="G2">
-        <v>-1.078</v>
-      </c>
-      <c r="H2">
-        <v>0.001605</v>
-      </c>
-      <c r="I2">
-        <v>0.5617</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>BFR_Post-Pre</t>
-        </is>
-      </c>
-      <c r="K2" t="b">
-        <v>1</v>
-      </c>
-      <c r="L2" t="b">
-        <v>0</v>
+        <v>0.981</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GOBP|GOBP_CARDIAC_CELL_DEVELOPMENT</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>GOBP</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>GOBP_CARDIAC_CELL_DEVELOPMENT</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Cardiac Cell
-Development</t>
-        </is>
+          <t>collapse survivors</t>
+        </is>
+      </c>
+      <c r="B3">
+        <v>126</v>
+      </c>
+      <c r="C3">
+        <v>126</v>
+      </c>
+      <c r="D3">
+        <v>3</v>
       </c>
       <c r="E3">
-        <v>29</v>
+        <v>0.861</v>
       </c>
       <c r="F3">
-        <v>-1.787</v>
+        <v>0</v>
       </c>
       <c r="G3">
-        <v>1.01</v>
-      </c>
-      <c r="H3">
-        <v>0.02478</v>
-      </c>
-      <c r="I3">
-        <v>0.7411</v>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>BFR_Post-Pre</t>
-        </is>
-      </c>
-      <c r="K3" t="b">
-        <v>1</v>
-      </c>
-      <c r="L3" t="b">
-        <v>0</v>
+        <v>0.976</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GOBP|GOBP_REGULATION_OF_PROTEIN_LOCALIZATION_TO_PLASMA_MEMBRANE</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>GOBP</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>GOBP_REGULATION_OF_PROTEIN_LOCALIZATION_TO_PLASMA_MEMBRANE</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Reg. PM Protein
-Localization</t>
-        </is>
+          <t>Hallmark and GO Slim</t>
+        </is>
+      </c>
+      <c r="B4">
+        <v>100</v>
+      </c>
+      <c r="C4">
+        <v>25</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
       </c>
       <c r="E4">
-        <v>41</v>
+        <v>0.8149999999999999</v>
       </c>
       <c r="F4">
-        <v>-1.735</v>
+        <v>0</v>
       </c>
       <c r="G4">
-        <v>1.012</v>
-      </c>
-      <c r="H4">
-        <v>0.04294</v>
-      </c>
-      <c r="I4">
-        <v>0.7226</v>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>BFR_Post-Pre</t>
-        </is>
-      </c>
-      <c r="K4" t="b">
-        <v>1</v>
-      </c>
-      <c r="L4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Reactome|REACTOME_REGULATION_OF_CDH1_POSTTRANSLATIONAL_PROCESSING_AND_TRAFFICKING_TO_PLASMA_MEMBRANE</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Reactome</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>REACTOME_REGULATION_OF_CDH1_POSTTRANSLATIONAL_PROCESSING_AND_TRAFFICKING_TO_PLASMA_MEMBRANE</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Reg. Cdh1
-Posttranslational
-Processing &amp;
-Trafficking To
-Plasma Membrane</t>
-        </is>
-      </c>
-      <c r="E5">
-        <v>18</v>
-      </c>
-      <c r="F5">
-        <v>-2.054</v>
-      </c>
-      <c r="G5">
-        <v>0.674</v>
-      </c>
-      <c r="H5">
-        <v>0.002907</v>
-      </c>
-      <c r="I5">
-        <v>0.9901</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>BFR_Post-Pre</t>
-        </is>
-      </c>
-      <c r="K5" t="b">
-        <v>1</v>
-      </c>
-      <c r="L5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>GOBP|GOBP_POSITIVE_REGULATION_OF_PROTEIN_LOCALIZATION_TO_MEMBRANE</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>GOBP</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>GOBP_POSITIVE_REGULATION_OF_PROTEIN_LOCALIZATION_TO_MEMBRANE</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Positive
-Reg. Protein
-Localization To
-Membrane</t>
-        </is>
-      </c>
-      <c r="E6">
-        <v>28</v>
-      </c>
-      <c r="F6">
-        <v>-1.733</v>
-      </c>
-      <c r="G6">
-        <v>0.854</v>
-      </c>
-      <c r="H6">
-        <v>0.03326</v>
-      </c>
-      <c r="I6">
-        <v>0.9032</v>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>BFR_Post-Pre</t>
-        </is>
-      </c>
-      <c r="K6" t="b">
-        <v>1</v>
-      </c>
-      <c r="L6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>GOBP|GOBP_REGULATION_OF_CELL_MORPHOGENESIS</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>GOBP</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>GOBP_REGULATION_OF_CELL_MORPHOGENESIS</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Reg. Cell
-Morphogenesis</t>
-        </is>
-      </c>
-      <c r="E7">
-        <v>48</v>
-      </c>
-      <c r="F7">
-        <v>-1.171</v>
-      </c>
-      <c r="G7">
-        <v>1.665</v>
-      </c>
-      <c r="H7">
-        <v>0.4341</v>
-      </c>
-      <c r="I7">
-        <v>0.04548</v>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>HLRT_Post-Pre</t>
-        </is>
-      </c>
-      <c r="K7" t="b">
-        <v>1</v>
-      </c>
-      <c r="L7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>GOBP|GOBP_REGULATION_OF_CELL_SHAPE</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>GOBP</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>GOBP_REGULATION_OF_CELL_SHAPE</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Reg. Cell Shape</t>
-        </is>
-      </c>
-      <c r="E8">
-        <v>30</v>
-      </c>
-      <c r="F8">
-        <v>-0.954</v>
-      </c>
-      <c r="G8">
-        <v>1.741</v>
-      </c>
-      <c r="H8">
-        <v>0.753</v>
-      </c>
-      <c r="I8">
-        <v>0.04778</v>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>HLRT_Post-Pre</t>
-        </is>
-      </c>
-      <c r="K8" t="b">
-        <v>1</v>
-      </c>
-      <c r="L8" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>GOBP|GOBP_POLYOL_METABOLIC_PROCESS</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>GOBP</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>GOBP_POLYOL_METABOLIC_PROCESS</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Polyol
-Metabolism</t>
-        </is>
-      </c>
-      <c r="E9">
-        <v>24</v>
-      </c>
-      <c r="F9">
-        <v>0.651</v>
-      </c>
-      <c r="G9">
-        <v>-1.748</v>
-      </c>
-      <c r="H9">
-        <v>0.9874000000000001</v>
-      </c>
-      <c r="I9">
-        <v>0.03191</v>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>HLRT_Post-Pre</t>
-        </is>
-      </c>
-      <c r="K9" t="b">
-        <v>1</v>
-      </c>
-      <c r="L9" t="b">
         <v>1</v>
       </c>
     </row>
@@ -944,6 +561,474 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:L9"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>set_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>database</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>pathway</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>label</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>genes</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>nes_x</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>nes_y</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>padj_x</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>padj_y</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>significance</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>discordant</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>survivor</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>GOBP|GOBP_SMALL_MOLECULE_CATABOLIC_PROCESS</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>GOBP</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>GOBP_SMALL_MOLECULE_CATABOLIC_PROCESS</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Small Molecule
+Catabolism</t>
+        </is>
+      </c>
+      <c r="E2">
+        <v>157</v>
+      </c>
+      <c r="F2">
+        <v>1.725</v>
+      </c>
+      <c r="G2">
+        <v>-1.078</v>
+      </c>
+      <c r="H2">
+        <v>0.001605</v>
+      </c>
+      <c r="I2">
+        <v>0.5617</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>BFR_Post-Pre</t>
+        </is>
+      </c>
+      <c r="K2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>GOBP|GOBP_CARDIAC_CELL_DEVELOPMENT</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>GOBP</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>GOBP_CARDIAC_CELL_DEVELOPMENT</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Cardiac Cell
+Development</t>
+        </is>
+      </c>
+      <c r="E3">
+        <v>29</v>
+      </c>
+      <c r="F3">
+        <v>-1.787</v>
+      </c>
+      <c r="G3">
+        <v>1.01</v>
+      </c>
+      <c r="H3">
+        <v>0.02478</v>
+      </c>
+      <c r="I3">
+        <v>0.7411</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>BFR_Post-Pre</t>
+        </is>
+      </c>
+      <c r="K3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>GOBP|GOBP_REGULATION_OF_PROTEIN_LOCALIZATION_TO_PLASMA_MEMBRANE</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>GOBP</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>GOBP_REGULATION_OF_PROTEIN_LOCALIZATION_TO_PLASMA_MEMBRANE</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Reg. PM Protein
+Localization</t>
+        </is>
+      </c>
+      <c r="E4">
+        <v>41</v>
+      </c>
+      <c r="F4">
+        <v>-1.735</v>
+      </c>
+      <c r="G4">
+        <v>1.012</v>
+      </c>
+      <c r="H4">
+        <v>0.04294</v>
+      </c>
+      <c r="I4">
+        <v>0.7226</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>BFR_Post-Pre</t>
+        </is>
+      </c>
+      <c r="K4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Reactome|REACTOME_REGULATION_OF_CDH1_POSTTRANSLATIONAL_PROCESSING_AND_TRAFFICKING_TO_PLASMA_MEMBRANE</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Reactome</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>REACTOME_REGULATION_OF_CDH1_POSTTRANSLATIONAL_PROCESSING_AND_TRAFFICKING_TO_PLASMA_MEMBRANE</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Reg. Cdh1
+Posttranslational
+Processing &amp;
+Trafficking To
+Plasma Membrane</t>
+        </is>
+      </c>
+      <c r="E5">
+        <v>18</v>
+      </c>
+      <c r="F5">
+        <v>-2.054</v>
+      </c>
+      <c r="G5">
+        <v>0.674</v>
+      </c>
+      <c r="H5">
+        <v>0.002907</v>
+      </c>
+      <c r="I5">
+        <v>0.9901</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>BFR_Post-Pre</t>
+        </is>
+      </c>
+      <c r="K5" t="b">
+        <v>1</v>
+      </c>
+      <c r="L5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>GOBP|GOBP_POSITIVE_REGULATION_OF_PROTEIN_LOCALIZATION_TO_MEMBRANE</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>GOBP</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>GOBP_POSITIVE_REGULATION_OF_PROTEIN_LOCALIZATION_TO_MEMBRANE</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Positive
+Reg. Protein
+Localization To
+Membrane</t>
+        </is>
+      </c>
+      <c r="E6">
+        <v>28</v>
+      </c>
+      <c r="F6">
+        <v>-1.733</v>
+      </c>
+      <c r="G6">
+        <v>0.854</v>
+      </c>
+      <c r="H6">
+        <v>0.03326</v>
+      </c>
+      <c r="I6">
+        <v>0.9032</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>BFR_Post-Pre</t>
+        </is>
+      </c>
+      <c r="K6" t="b">
+        <v>1</v>
+      </c>
+      <c r="L6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>GOBP|GOBP_REGULATION_OF_CELL_MORPHOGENESIS</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>GOBP</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>GOBP_REGULATION_OF_CELL_MORPHOGENESIS</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Reg. Cell
+Morphogenesis</t>
+        </is>
+      </c>
+      <c r="E7">
+        <v>48</v>
+      </c>
+      <c r="F7">
+        <v>-1.171</v>
+      </c>
+      <c r="G7">
+        <v>1.665</v>
+      </c>
+      <c r="H7">
+        <v>0.4341</v>
+      </c>
+      <c r="I7">
+        <v>0.04548</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>HLRT_Post-Pre</t>
+        </is>
+      </c>
+      <c r="K7" t="b">
+        <v>1</v>
+      </c>
+      <c r="L7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>GOBP|GOBP_REGULATION_OF_CELL_SHAPE</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>GOBP</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>GOBP_REGULATION_OF_CELL_SHAPE</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Reg. Cell Shape</t>
+        </is>
+      </c>
+      <c r="E8">
+        <v>30</v>
+      </c>
+      <c r="F8">
+        <v>-0.954</v>
+      </c>
+      <c r="G8">
+        <v>1.741</v>
+      </c>
+      <c r="H8">
+        <v>0.753</v>
+      </c>
+      <c r="I8">
+        <v>0.04778</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>HLRT_Post-Pre</t>
+        </is>
+      </c>
+      <c r="K8" t="b">
+        <v>1</v>
+      </c>
+      <c r="L8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>GOBP|GOBP_POLYOL_METABOLIC_PROCESS</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>GOBP</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>GOBP_POLYOL_METABOLIC_PROCESS</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Polyol
+Metabolism</t>
+        </is>
+      </c>
+      <c r="E9">
+        <v>24</v>
+      </c>
+      <c r="F9">
+        <v>0.651</v>
+      </c>
+      <c r="G9">
+        <v>-1.748</v>
+      </c>
+      <c r="H9">
+        <v>0.9874000000000001</v>
+      </c>
+      <c r="I9">
+        <v>0.03191</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>HLRT_Post-Pre</t>
+        </is>
+      </c>
+      <c r="K9" t="b">
+        <v>1</v>
+      </c>
+      <c r="L9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L1991"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -99634,154 +99719,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>input</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>path</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>md5</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>set_tests</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>03_Pathway_Enrichment/01_run_fgsea_and_fry/c_data/set_tests.rds</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>192186238ddf41bd2ee16caee3a2c5f0</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>package</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>version</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>here</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>1.0.2</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>fgsea</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>1.38.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>dplyr</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>1.2.1</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>ggplot2</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>4.0.3</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>ggrepel</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>0.9.8</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>patchwork</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>1.3.2</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>enrichVolcano</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>0.3.0.9000</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
move the pathway tables into one workbook per step and the figures onto captioned S1-S19 pages
The seven steps read each other's outputs, so they change together.
- gene_sets.rds keeps only the set list; the catalogue and protein map move to the workbook.
- fgsea and fry write one workbook instead of an rds, a csv and a workbook.
- The volcanoes ring the top 12 sets, lose their NA subtitles, and point leading-edge ticks at
  the protein fgsea ranked.
- The NES scatter counts its discordant sets instead of saying eight.
- singscore writes its matrix to set_scores.rds for 05, since a trip through Excel breaks its
  rank ties.
- Classify and associate inlines its single-use helpers and builds one chance table.
- Input checksums, package-version sheets, timestamps and the combined-PDF step go.
</commit_message>
<xml_diff>
--- a/03_Pathway_Enrichment/03_enrich_scatter_fgsea/c_data/03_enrich_scatter_fgsea.xlsx
+++ b/03_Pathway_Enrichment/03_enrich_scatter_fgsea/c_data/03_enrich_scatter_fgsea.xlsx
@@ -7,11 +7,10 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="concordance" sheetId="1" r:id="rId1"/>
-    <sheet name="discordant" sheetId="2" r:id="rId2"/>
-    <sheet name="nes_scatter" sheetId="3" r:id="rId3"/>
-    <sheet name="input_manifest" sheetId="4" r:id="rId4"/>
-    <sheet name="package_versions" sheetId="5" r:id="rId5"/>
+    <sheet name="overview" sheetId="1" r:id="rId1"/>
+    <sheet name="concordance" sheetId="2" r:id="rId2"/>
+    <sheet name="discordant" sheetId="3" r:id="rId3"/>
+    <sheet name="nes_scatter" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -355,119 +354,83 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>population</t>
+          <t>sheet</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>sets</t>
+          <t>rows</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>significant</t>
+          <t>columns</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>discordant</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>rho</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>p</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>same_sign</t>
+          <t>description</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>all collections</t>
+          <t>concordance</t>
         </is>
       </c>
       <c r="B2">
-        <v>1990</v>
+        <v>3</v>
       </c>
       <c r="C2">
-        <v>418</v>
-      </c>
-      <c r="D2">
-        <v>8</v>
-      </c>
-      <c r="E2">
-        <v>0.827</v>
-      </c>
-      <c r="F2">
-        <v>0</v>
-      </c>
-      <c r="G2">
-        <v>0.981</v>
+        <v>7</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Spearman rho and sign agreement of NES between the two training contrasts, per population</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>collapse survivors</t>
+          <t>discordant</t>
         </is>
       </c>
       <c r="B3">
-        <v>126</v>
+        <v>8</v>
       </c>
       <c r="C3">
-        <v>126</v>
-      </c>
-      <c r="D3">
-        <v>3</v>
-      </c>
-      <c r="E3">
-        <v>0.861</v>
-      </c>
-      <c r="F3">
-        <v>0</v>
-      </c>
-      <c r="G3">
-        <v>0.976</v>
+        <v>12</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Sets significant in one arm with NES of opposite sign in the other</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Hallmark and GO Slim</t>
+          <t>nes_scatter</t>
         </is>
       </c>
       <c r="B4">
-        <v>100</v>
+        <v>1990</v>
       </c>
       <c r="C4">
-        <v>25</v>
-      </c>
-      <c r="D4">
-        <v>0</v>
-      </c>
-      <c r="E4">
-        <v>0.8149999999999999</v>
-      </c>
-      <c r="F4">
-        <v>0</v>
-      </c>
-      <c r="G4">
-        <v>1</v>
+        <v>12</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Every set with its NES and adjusted p in both training contrasts</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -477,464 +440,118 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>set_id</t>
+          <t>population</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>database</t>
+          <t>sets</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>pathway</t>
+          <t>significant</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>label</t>
+          <t>discordant</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>genes</t>
+          <t>rho</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>nes_x</t>
+          <t>p</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>nes_y</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>padj_x</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>padj_y</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>significance</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>discordant</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>survivor</t>
+          <t>same_sign</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>GOBP|GOBP_SMALL_MOLECULE_CATABOLIC_PROCESS</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>GOBP</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>GOBP_SMALL_MOLECULE_CATABOLIC_PROCESS</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Small Molecule
-Catabolism</t>
-        </is>
+          <t>all collections</t>
+        </is>
+      </c>
+      <c r="B2">
+        <v>1990</v>
+      </c>
+      <c r="C2">
+        <v>418</v>
+      </c>
+      <c r="D2">
+        <v>8</v>
       </c>
       <c r="E2">
-        <v>157</v>
+        <v>0.827</v>
       </c>
       <c r="F2">
-        <v>1.725</v>
+        <v>0</v>
       </c>
       <c r="G2">
-        <v>-1.078</v>
-      </c>
-      <c r="H2">
-        <v>0.001605</v>
-      </c>
-      <c r="I2">
-        <v>0.5617</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>BFR_Post-Pre</t>
-        </is>
-      </c>
-      <c r="K2" t="b">
-        <v>1</v>
-      </c>
-      <c r="L2" t="b">
-        <v>0</v>
+        <v>0.981</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GOBP|GOBP_CARDIAC_CELL_DEVELOPMENT</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>GOBP</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>GOBP_CARDIAC_CELL_DEVELOPMENT</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Cardiac Cell
-Development</t>
-        </is>
+          <t>collapse survivors</t>
+        </is>
+      </c>
+      <c r="B3">
+        <v>126</v>
+      </c>
+      <c r="C3">
+        <v>126</v>
+      </c>
+      <c r="D3">
+        <v>3</v>
       </c>
       <c r="E3">
-        <v>29</v>
+        <v>0.861</v>
       </c>
       <c r="F3">
-        <v>-1.787</v>
+        <v>0</v>
       </c>
       <c r="G3">
-        <v>1.01</v>
-      </c>
-      <c r="H3">
-        <v>0.02478</v>
-      </c>
-      <c r="I3">
-        <v>0.7411</v>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>BFR_Post-Pre</t>
-        </is>
-      </c>
-      <c r="K3" t="b">
-        <v>1</v>
-      </c>
-      <c r="L3" t="b">
-        <v>0</v>
+        <v>0.976</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GOBP|GOBP_REGULATION_OF_PROTEIN_LOCALIZATION_TO_PLASMA_MEMBRANE</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>GOBP</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>GOBP_REGULATION_OF_PROTEIN_LOCALIZATION_TO_PLASMA_MEMBRANE</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Reg. PM Protein
-Localization</t>
-        </is>
+          <t>Hallmark and GO Slim</t>
+        </is>
+      </c>
+      <c r="B4">
+        <v>100</v>
+      </c>
+      <c r="C4">
+        <v>25</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
       </c>
       <c r="E4">
-        <v>41</v>
+        <v>0.8149999999999999</v>
       </c>
       <c r="F4">
-        <v>-1.735</v>
+        <v>0</v>
       </c>
       <c r="G4">
-        <v>1.012</v>
-      </c>
-      <c r="H4">
-        <v>0.04294</v>
-      </c>
-      <c r="I4">
-        <v>0.7226</v>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>BFR_Post-Pre</t>
-        </is>
-      </c>
-      <c r="K4" t="b">
-        <v>1</v>
-      </c>
-      <c r="L4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Reactome|REACTOME_REGULATION_OF_CDH1_POSTTRANSLATIONAL_PROCESSING_AND_TRAFFICKING_TO_PLASMA_MEMBRANE</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Reactome</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>REACTOME_REGULATION_OF_CDH1_POSTTRANSLATIONAL_PROCESSING_AND_TRAFFICKING_TO_PLASMA_MEMBRANE</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Reg. Cdh1
-Posttranslational
-Processing &amp;
-Trafficking To
-Plasma Membrane</t>
-        </is>
-      </c>
-      <c r="E5">
-        <v>18</v>
-      </c>
-      <c r="F5">
-        <v>-2.054</v>
-      </c>
-      <c r="G5">
-        <v>0.674</v>
-      </c>
-      <c r="H5">
-        <v>0.002907</v>
-      </c>
-      <c r="I5">
-        <v>0.9901</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>BFR_Post-Pre</t>
-        </is>
-      </c>
-      <c r="K5" t="b">
-        <v>1</v>
-      </c>
-      <c r="L5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>GOBP|GOBP_POSITIVE_REGULATION_OF_PROTEIN_LOCALIZATION_TO_MEMBRANE</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>GOBP</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>GOBP_POSITIVE_REGULATION_OF_PROTEIN_LOCALIZATION_TO_MEMBRANE</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Positive
-Reg. Protein
-Localization To
-Membrane</t>
-        </is>
-      </c>
-      <c r="E6">
-        <v>28</v>
-      </c>
-      <c r="F6">
-        <v>-1.733</v>
-      </c>
-      <c r="G6">
-        <v>0.854</v>
-      </c>
-      <c r="H6">
-        <v>0.03326</v>
-      </c>
-      <c r="I6">
-        <v>0.9032</v>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>BFR_Post-Pre</t>
-        </is>
-      </c>
-      <c r="K6" t="b">
-        <v>1</v>
-      </c>
-      <c r="L6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>GOBP|GOBP_REGULATION_OF_CELL_MORPHOGENESIS</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>GOBP</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>GOBP_REGULATION_OF_CELL_MORPHOGENESIS</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Reg. Cell
-Morphogenesis</t>
-        </is>
-      </c>
-      <c r="E7">
-        <v>48</v>
-      </c>
-      <c r="F7">
-        <v>-1.171</v>
-      </c>
-      <c r="G7">
-        <v>1.665</v>
-      </c>
-      <c r="H7">
-        <v>0.4341</v>
-      </c>
-      <c r="I7">
-        <v>0.04548</v>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>HLRT_Post-Pre</t>
-        </is>
-      </c>
-      <c r="K7" t="b">
-        <v>1</v>
-      </c>
-      <c r="L7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>GOBP|GOBP_REGULATION_OF_CELL_SHAPE</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>GOBP</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>GOBP_REGULATION_OF_CELL_SHAPE</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Reg. Cell Shape</t>
-        </is>
-      </c>
-      <c r="E8">
-        <v>30</v>
-      </c>
-      <c r="F8">
-        <v>-0.954</v>
-      </c>
-      <c r="G8">
-        <v>1.741</v>
-      </c>
-      <c r="H8">
-        <v>0.753</v>
-      </c>
-      <c r="I8">
-        <v>0.04778</v>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>HLRT_Post-Pre</t>
-        </is>
-      </c>
-      <c r="K8" t="b">
-        <v>1</v>
-      </c>
-      <c r="L8" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>GOBP|GOBP_POLYOL_METABOLIC_PROCESS</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>GOBP</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>GOBP_POLYOL_METABOLIC_PROCESS</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Polyol
-Metabolism</t>
-        </is>
-      </c>
-      <c r="E9">
-        <v>24</v>
-      </c>
-      <c r="F9">
-        <v>0.651</v>
-      </c>
-      <c r="G9">
-        <v>-1.748</v>
-      </c>
-      <c r="H9">
-        <v>0.9874000000000001</v>
-      </c>
-      <c r="I9">
-        <v>0.03191</v>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>HLRT_Post-Pre</t>
-        </is>
-      </c>
-      <c r="K9" t="b">
-        <v>1</v>
-      </c>
-      <c r="L9" t="b">
         <v>1</v>
       </c>
     </row>
@@ -944,6 +561,474 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:L9"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>set_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>database</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>pathway</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>label</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>genes</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>nes_x</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>nes_y</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>padj_x</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>padj_y</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>significance</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>discordant</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>survivor</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>GOBP|GOBP_SMALL_MOLECULE_CATABOLIC_PROCESS</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>GOBP</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>GOBP_SMALL_MOLECULE_CATABOLIC_PROCESS</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Small Molecule
+Catabolism</t>
+        </is>
+      </c>
+      <c r="E2">
+        <v>157</v>
+      </c>
+      <c r="F2">
+        <v>1.725</v>
+      </c>
+      <c r="G2">
+        <v>-1.078</v>
+      </c>
+      <c r="H2">
+        <v>0.001605</v>
+      </c>
+      <c r="I2">
+        <v>0.5617</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>BFR_Post-Pre</t>
+        </is>
+      </c>
+      <c r="K2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>GOBP|GOBP_CARDIAC_CELL_DEVELOPMENT</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>GOBP</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>GOBP_CARDIAC_CELL_DEVELOPMENT</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Cardiac Cell
+Development</t>
+        </is>
+      </c>
+      <c r="E3">
+        <v>29</v>
+      </c>
+      <c r="F3">
+        <v>-1.787</v>
+      </c>
+      <c r="G3">
+        <v>1.01</v>
+      </c>
+      <c r="H3">
+        <v>0.02478</v>
+      </c>
+      <c r="I3">
+        <v>0.7411</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>BFR_Post-Pre</t>
+        </is>
+      </c>
+      <c r="K3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>GOBP|GOBP_REGULATION_OF_PROTEIN_LOCALIZATION_TO_PLASMA_MEMBRANE</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>GOBP</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>GOBP_REGULATION_OF_PROTEIN_LOCALIZATION_TO_PLASMA_MEMBRANE</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Reg. PM Protein
+Localization</t>
+        </is>
+      </c>
+      <c r="E4">
+        <v>41</v>
+      </c>
+      <c r="F4">
+        <v>-1.735</v>
+      </c>
+      <c r="G4">
+        <v>1.012</v>
+      </c>
+      <c r="H4">
+        <v>0.04294</v>
+      </c>
+      <c r="I4">
+        <v>0.7226</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>BFR_Post-Pre</t>
+        </is>
+      </c>
+      <c r="K4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Reactome|REACTOME_REGULATION_OF_CDH1_POSTTRANSLATIONAL_PROCESSING_AND_TRAFFICKING_TO_PLASMA_MEMBRANE</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Reactome</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>REACTOME_REGULATION_OF_CDH1_POSTTRANSLATIONAL_PROCESSING_AND_TRAFFICKING_TO_PLASMA_MEMBRANE</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Reg. Cdh1
+Posttranslational
+Processing &amp;
+Trafficking To
+Plasma Membrane</t>
+        </is>
+      </c>
+      <c r="E5">
+        <v>18</v>
+      </c>
+      <c r="F5">
+        <v>-2.054</v>
+      </c>
+      <c r="G5">
+        <v>0.674</v>
+      </c>
+      <c r="H5">
+        <v>0.002907</v>
+      </c>
+      <c r="I5">
+        <v>0.9901</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>BFR_Post-Pre</t>
+        </is>
+      </c>
+      <c r="K5" t="b">
+        <v>1</v>
+      </c>
+      <c r="L5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>GOBP|GOBP_POSITIVE_REGULATION_OF_PROTEIN_LOCALIZATION_TO_MEMBRANE</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>GOBP</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>GOBP_POSITIVE_REGULATION_OF_PROTEIN_LOCALIZATION_TO_MEMBRANE</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Positive
+Reg. Protein
+Localization To
+Membrane</t>
+        </is>
+      </c>
+      <c r="E6">
+        <v>28</v>
+      </c>
+      <c r="F6">
+        <v>-1.733</v>
+      </c>
+      <c r="G6">
+        <v>0.854</v>
+      </c>
+      <c r="H6">
+        <v>0.03326</v>
+      </c>
+      <c r="I6">
+        <v>0.9032</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>BFR_Post-Pre</t>
+        </is>
+      </c>
+      <c r="K6" t="b">
+        <v>1</v>
+      </c>
+      <c r="L6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>GOBP|GOBP_REGULATION_OF_CELL_MORPHOGENESIS</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>GOBP</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>GOBP_REGULATION_OF_CELL_MORPHOGENESIS</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Reg. Cell
+Morphogenesis</t>
+        </is>
+      </c>
+      <c r="E7">
+        <v>48</v>
+      </c>
+      <c r="F7">
+        <v>-1.171</v>
+      </c>
+      <c r="G7">
+        <v>1.665</v>
+      </c>
+      <c r="H7">
+        <v>0.4341</v>
+      </c>
+      <c r="I7">
+        <v>0.04548</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>HLRT_Post-Pre</t>
+        </is>
+      </c>
+      <c r="K7" t="b">
+        <v>1</v>
+      </c>
+      <c r="L7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>GOBP|GOBP_REGULATION_OF_CELL_SHAPE</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>GOBP</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>GOBP_REGULATION_OF_CELL_SHAPE</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Reg. Cell Shape</t>
+        </is>
+      </c>
+      <c r="E8">
+        <v>30</v>
+      </c>
+      <c r="F8">
+        <v>-0.954</v>
+      </c>
+      <c r="G8">
+        <v>1.741</v>
+      </c>
+      <c r="H8">
+        <v>0.753</v>
+      </c>
+      <c r="I8">
+        <v>0.04778</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>HLRT_Post-Pre</t>
+        </is>
+      </c>
+      <c r="K8" t="b">
+        <v>1</v>
+      </c>
+      <c r="L8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>GOBP|GOBP_POLYOL_METABOLIC_PROCESS</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>GOBP</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>GOBP_POLYOL_METABOLIC_PROCESS</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Polyol
+Metabolism</t>
+        </is>
+      </c>
+      <c r="E9">
+        <v>24</v>
+      </c>
+      <c r="F9">
+        <v>0.651</v>
+      </c>
+      <c r="G9">
+        <v>-1.748</v>
+      </c>
+      <c r="H9">
+        <v>0.9874000000000001</v>
+      </c>
+      <c r="I9">
+        <v>0.03191</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>HLRT_Post-Pre</t>
+        </is>
+      </c>
+      <c r="K9" t="b">
+        <v>1</v>
+      </c>
+      <c r="L9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L1991"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -99634,154 +99719,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>input</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>path</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>md5</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>set_tests</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>03_Pathway_Enrichment/01_run_fgsea_and_fry/c_data/set_tests.rds</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>192186238ddf41bd2ee16caee3a2c5f0</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>package</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>version</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>here</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>1.0.2</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>fgsea</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>1.38.0</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>dplyr</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>1.2.1</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>ggplot2</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>4.0.3</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>ggrepel</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>0.9.8</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>patchwork</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>1.3.2</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>enrichVolcano</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>0.3.0.9000</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Fix stage 03 captions and chance ratios, remove duplicate GSEA run
</commit_message>
<xml_diff>
--- a/03_Pathway_Enrichment/03_enrich_scatter_fgsea/c_data/03_enrich_scatter_fgsea.xlsx
+++ b/03_Pathway_Enrichment/03_enrich_scatter_fgsea/c_data/03_enrich_scatter_fgsea.xlsx
@@ -7,10 +7,9 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="overview" sheetId="1" r:id="rId1"/>
-    <sheet name="concordance" sheetId="2" r:id="rId2"/>
-    <sheet name="discordant" sheetId="3" r:id="rId3"/>
-    <sheet name="nes_scatter" sheetId="4" r:id="rId4"/>
+    <sheet name="concordance" sheetId="1" r:id="rId1"/>
+    <sheet name="discordant" sheetId="2" r:id="rId2"/>
+    <sheet name="nes_scatter" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -354,83 +353,119 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>sheet</t>
+          <t>population</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>rows</t>
+          <t>sets</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>columns</t>
+          <t>significant</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>discordant</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>rho</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>p</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>same_sign</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>concordance</t>
+          <t>all collections</t>
         </is>
       </c>
       <c r="B2">
-        <v>3</v>
+        <v>1990</v>
       </c>
       <c r="C2">
-        <v>7</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>NES agreement between training contrasts</t>
-        </is>
+        <v>418</v>
+      </c>
+      <c r="D2">
+        <v>8</v>
+      </c>
+      <c r="E2">
+        <v>0.827</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>0.981</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>discordant</t>
+          <t>collapse survivors</t>
         </is>
       </c>
       <c r="B3">
-        <v>8</v>
+        <v>126</v>
       </c>
       <c r="C3">
-        <v>12</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Sets with opposite NES signs</t>
-        </is>
+        <v>126</v>
+      </c>
+      <c r="D3">
+        <v>3</v>
+      </c>
+      <c r="E3">
+        <v>0.861</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>0.976</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>nes_scatter</t>
+          <t>Hallmark and GO Slim</t>
         </is>
       </c>
       <c r="B4">
-        <v>1990</v>
+        <v>100</v>
       </c>
       <c r="C4">
-        <v>12</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>NES and adjusted p, both contrasts</t>
-        </is>
+        <v>25</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0.8149999999999999</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -440,118 +475,472 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>population</t>
+          <t>set_id</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>sets</t>
+          <t>database</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>significant</t>
+          <t>pathway</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>label</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>genes</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>nes_x</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>nes_y</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>padj_x</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>padj_y</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>significance</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>discordant</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>rho</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>p</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>same_sign</t>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>survivor</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>all collections</t>
-        </is>
-      </c>
-      <c r="B2">
-        <v>1990</v>
-      </c>
-      <c r="C2">
-        <v>418</v>
-      </c>
-      <c r="D2">
-        <v>8</v>
+          <t>GOBP|GOBP_SMALL_MOLECULE_CATABOLIC_PROCESS</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>GOBP</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>GOBP_SMALL_MOLECULE_CATABOLIC_PROCESS</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Small Molecule
+Catabolic
+Process</t>
+        </is>
       </c>
       <c r="E2">
-        <v>0.827</v>
+        <v>157</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>1.725</v>
       </c>
       <c r="G2">
-        <v>0.981</v>
+        <v>-1.078</v>
+      </c>
+      <c r="H2">
+        <v>0.001605</v>
+      </c>
+      <c r="I2">
+        <v>0.5617</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>BFR_Post-Pre</t>
+        </is>
+      </c>
+      <c r="K2" t="b">
+        <v>1</v>
+      </c>
+      <c r="L2" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>collapse survivors</t>
-        </is>
-      </c>
-      <c r="B3">
-        <v>126</v>
-      </c>
-      <c r="C3">
-        <v>126</v>
-      </c>
-      <c r="D3">
-        <v>3</v>
+          <t>GOBP|GOBP_CARDIAC_CELL_DEVELOPMENT</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>GOBP</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>GOBP_CARDIAC_CELL_DEVELOPMENT</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Cardiac Cell
+Development</t>
+        </is>
       </c>
       <c r="E3">
-        <v>0.861</v>
+        <v>29</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>-1.787</v>
       </c>
       <c r="G3">
-        <v>0.976</v>
+        <v>1.01</v>
+      </c>
+      <c r="H3">
+        <v>0.02478</v>
+      </c>
+      <c r="I3">
+        <v>0.7411</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>BFR_Post-Pre</t>
+        </is>
+      </c>
+      <c r="K3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L3" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Hallmark and GO Slim</t>
-        </is>
-      </c>
-      <c r="B4">
-        <v>100</v>
-      </c>
-      <c r="C4">
-        <v>25</v>
-      </c>
-      <c r="D4">
-        <v>0</v>
+          <t>GOBP|GOBP_REGULATION_OF_PROTEIN_LOCALIZATION_TO_PLASMA_MEMBRANE</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>GOBP</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>GOBP_REGULATION_OF_PROTEIN_LOCALIZATION_TO_PLASMA_MEMBRANE</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Regulation
+Of Protein
+Localization To
+Plasma Membrane</t>
+        </is>
       </c>
       <c r="E4">
-        <v>0.8149999999999999</v>
+        <v>41</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>-1.735</v>
       </c>
       <c r="G4">
+        <v>1.012</v>
+      </c>
+      <c r="H4">
+        <v>0.04294</v>
+      </c>
+      <c r="I4">
+        <v>0.7226</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>BFR_Post-Pre</t>
+        </is>
+      </c>
+      <c r="K4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Reactome|REACTOME_REGULATION_OF_CDH1_POSTTRANSLATIONAL_PROCESSING_AND_TRAFFICKING_TO_PLASMA_MEMBRANE</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Reactome</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>REACTOME_REGULATION_OF_CDH1_POSTTRANSLATIONAL_PROCESSING_AND_TRAFFICKING_TO_PLASMA_MEMBRANE</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Regulation
+Of Cdh1
+Posttranslational
+Processing And
+Trafficking To
+Plasma Membrane</t>
+        </is>
+      </c>
+      <c r="E5">
+        <v>18</v>
+      </c>
+      <c r="F5">
+        <v>-2.054</v>
+      </c>
+      <c r="G5">
+        <v>0.674</v>
+      </c>
+      <c r="H5">
+        <v>0.002907</v>
+      </c>
+      <c r="I5">
+        <v>0.9901</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>BFR_Post-Pre</t>
+        </is>
+      </c>
+      <c r="K5" t="b">
+        <v>1</v>
+      </c>
+      <c r="L5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>GOBP|GOBP_POSITIVE_REGULATION_OF_PROTEIN_LOCALIZATION_TO_MEMBRANE</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>GOBP</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>GOBP_POSITIVE_REGULATION_OF_PROTEIN_LOCALIZATION_TO_MEMBRANE</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Positive
+Regulation
+Of Protein
+Localization To
+Membrane</t>
+        </is>
+      </c>
+      <c r="E6">
+        <v>28</v>
+      </c>
+      <c r="F6">
+        <v>-1.733</v>
+      </c>
+      <c r="G6">
+        <v>0.854</v>
+      </c>
+      <c r="H6">
+        <v>0.03326</v>
+      </c>
+      <c r="I6">
+        <v>0.9032</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>BFR_Post-Pre</t>
+        </is>
+      </c>
+      <c r="K6" t="b">
+        <v>1</v>
+      </c>
+      <c r="L6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>GOBP|GOBP_REGULATION_OF_CELL_MORPHOGENESIS</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>GOBP</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>GOBP_REGULATION_OF_CELL_MORPHOGENESIS</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Regulation
+Of Cell
+Morphogenesis</t>
+        </is>
+      </c>
+      <c r="E7">
+        <v>48</v>
+      </c>
+      <c r="F7">
+        <v>-1.171</v>
+      </c>
+      <c r="G7">
+        <v>1.665</v>
+      </c>
+      <c r="H7">
+        <v>0.4341</v>
+      </c>
+      <c r="I7">
+        <v>0.04548</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>HLRT_Post-Pre</t>
+        </is>
+      </c>
+      <c r="K7" t="b">
+        <v>1</v>
+      </c>
+      <c r="L7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>GOBP|GOBP_REGULATION_OF_CELL_SHAPE</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>GOBP</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>GOBP_REGULATION_OF_CELL_SHAPE</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Regulation Of
+Cell Shape</t>
+        </is>
+      </c>
+      <c r="E8">
+        <v>30</v>
+      </c>
+      <c r="F8">
+        <v>-0.954</v>
+      </c>
+      <c r="G8">
+        <v>1.741</v>
+      </c>
+      <c r="H8">
+        <v>0.753</v>
+      </c>
+      <c r="I8">
+        <v>0.04778</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>HLRT_Post-Pre</t>
+        </is>
+      </c>
+      <c r="K8" t="b">
+        <v>1</v>
+      </c>
+      <c r="L8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>GOBP|GOBP_POLYOL_METABOLIC_PROCESS</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>GOBP</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>GOBP_POLYOL_METABOLIC_PROCESS</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Polyol
+Metabolic
+Process</t>
+        </is>
+      </c>
+      <c r="E9">
+        <v>24</v>
+      </c>
+      <c r="F9">
+        <v>0.651</v>
+      </c>
+      <c r="G9">
+        <v>-1.748</v>
+      </c>
+      <c r="H9">
+        <v>0.9874000000000001</v>
+      </c>
+      <c r="I9">
+        <v>0.03191</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>HLRT_Post-Pre</t>
+        </is>
+      </c>
+      <c r="K9" t="b">
+        <v>1</v>
+      </c>
+      <c r="L9" t="b">
         <v>1</v>
       </c>
     </row>
@@ -561,482 +950,6 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L9"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>set_id</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>database</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>pathway</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>label</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>genes</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>nes_x</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>nes_y</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>padj_x</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>padj_y</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>significance</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>discordant</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>survivor</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>GOBP|GOBP_SMALL_MOLECULE_CATABOLIC_PROCESS</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>GOBP</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>GOBP_SMALL_MOLECULE_CATABOLIC_PROCESS</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Small Molecule
-Catabolic
-Process</t>
-        </is>
-      </c>
-      <c r="E2">
-        <v>157</v>
-      </c>
-      <c r="F2">
-        <v>1.725</v>
-      </c>
-      <c r="G2">
-        <v>-1.078</v>
-      </c>
-      <c r="H2">
-        <v>0.001605</v>
-      </c>
-      <c r="I2">
-        <v>0.5617</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>BFR_Post-Pre</t>
-        </is>
-      </c>
-      <c r="K2" t="b">
-        <v>1</v>
-      </c>
-      <c r="L2" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>GOBP|GOBP_CARDIAC_CELL_DEVELOPMENT</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>GOBP</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>GOBP_CARDIAC_CELL_DEVELOPMENT</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Cardiac Cell
-Development</t>
-        </is>
-      </c>
-      <c r="E3">
-        <v>29</v>
-      </c>
-      <c r="F3">
-        <v>-1.787</v>
-      </c>
-      <c r="G3">
-        <v>1.01</v>
-      </c>
-      <c r="H3">
-        <v>0.02478</v>
-      </c>
-      <c r="I3">
-        <v>0.7411</v>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>BFR_Post-Pre</t>
-        </is>
-      </c>
-      <c r="K3" t="b">
-        <v>1</v>
-      </c>
-      <c r="L3" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>GOBP|GOBP_REGULATION_OF_PROTEIN_LOCALIZATION_TO_PLASMA_MEMBRANE</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>GOBP</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>GOBP_REGULATION_OF_PROTEIN_LOCALIZATION_TO_PLASMA_MEMBRANE</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Regulation
-Of Protein
-Localization To
-Plasma Membrane</t>
-        </is>
-      </c>
-      <c r="E4">
-        <v>41</v>
-      </c>
-      <c r="F4">
-        <v>-1.735</v>
-      </c>
-      <c r="G4">
-        <v>1.012</v>
-      </c>
-      <c r="H4">
-        <v>0.04294</v>
-      </c>
-      <c r="I4">
-        <v>0.7226</v>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>BFR_Post-Pre</t>
-        </is>
-      </c>
-      <c r="K4" t="b">
-        <v>1</v>
-      </c>
-      <c r="L4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Reactome|REACTOME_REGULATION_OF_CDH1_POSTTRANSLATIONAL_PROCESSING_AND_TRAFFICKING_TO_PLASMA_MEMBRANE</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Reactome</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>REACTOME_REGULATION_OF_CDH1_POSTTRANSLATIONAL_PROCESSING_AND_TRAFFICKING_TO_PLASMA_MEMBRANE</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Regulation
-Of Cdh1
-Posttranslational
-Processing And
-Trafficking To
-Plasma Membrane</t>
-        </is>
-      </c>
-      <c r="E5">
-        <v>18</v>
-      </c>
-      <c r="F5">
-        <v>-2.054</v>
-      </c>
-      <c r="G5">
-        <v>0.674</v>
-      </c>
-      <c r="H5">
-        <v>0.002907</v>
-      </c>
-      <c r="I5">
-        <v>0.9901</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>BFR_Post-Pre</t>
-        </is>
-      </c>
-      <c r="K5" t="b">
-        <v>1</v>
-      </c>
-      <c r="L5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>GOBP|GOBP_POSITIVE_REGULATION_OF_PROTEIN_LOCALIZATION_TO_MEMBRANE</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>GOBP</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>GOBP_POSITIVE_REGULATION_OF_PROTEIN_LOCALIZATION_TO_MEMBRANE</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Positive
-Regulation
-Of Protein
-Localization To
-Membrane</t>
-        </is>
-      </c>
-      <c r="E6">
-        <v>28</v>
-      </c>
-      <c r="F6">
-        <v>-1.733</v>
-      </c>
-      <c r="G6">
-        <v>0.854</v>
-      </c>
-      <c r="H6">
-        <v>0.03326</v>
-      </c>
-      <c r="I6">
-        <v>0.9032</v>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>BFR_Post-Pre</t>
-        </is>
-      </c>
-      <c r="K6" t="b">
-        <v>1</v>
-      </c>
-      <c r="L6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>GOBP|GOBP_REGULATION_OF_CELL_MORPHOGENESIS</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>GOBP</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>GOBP_REGULATION_OF_CELL_MORPHOGENESIS</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Regulation
-Of Cell
-Morphogenesis</t>
-        </is>
-      </c>
-      <c r="E7">
-        <v>48</v>
-      </c>
-      <c r="F7">
-        <v>-1.171</v>
-      </c>
-      <c r="G7">
-        <v>1.665</v>
-      </c>
-      <c r="H7">
-        <v>0.4341</v>
-      </c>
-      <c r="I7">
-        <v>0.04548</v>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>HLRT_Post-Pre</t>
-        </is>
-      </c>
-      <c r="K7" t="b">
-        <v>1</v>
-      </c>
-      <c r="L7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>GOBP|GOBP_REGULATION_OF_CELL_SHAPE</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>GOBP</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>GOBP_REGULATION_OF_CELL_SHAPE</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Regulation Of
-Cell Shape</t>
-        </is>
-      </c>
-      <c r="E8">
-        <v>30</v>
-      </c>
-      <c r="F8">
-        <v>-0.954</v>
-      </c>
-      <c r="G8">
-        <v>1.741</v>
-      </c>
-      <c r="H8">
-        <v>0.753</v>
-      </c>
-      <c r="I8">
-        <v>0.04778</v>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>HLRT_Post-Pre</t>
-        </is>
-      </c>
-      <c r="K8" t="b">
-        <v>1</v>
-      </c>
-      <c r="L8" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>GOBP|GOBP_POLYOL_METABOLIC_PROCESS</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>GOBP</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>GOBP_POLYOL_METABOLIC_PROCESS</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Polyol
-Metabolic
-Process</t>
-        </is>
-      </c>
-      <c r="E9">
-        <v>24</v>
-      </c>
-      <c r="F9">
-        <v>0.651</v>
-      </c>
-      <c r="G9">
-        <v>-1.748</v>
-      </c>
-      <c r="H9">
-        <v>0.9874000000000001</v>
-      </c>
-      <c r="I9">
-        <v>0.03191</v>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>HLRT_Post-Pre</t>
-        </is>
-      </c>
-      <c r="K9" t="b">
-        <v>1</v>
-      </c>
-      <c r="L9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L1991"/>
   <sheetFormatPr defaultRowHeight="15"/>

</xml_diff>